<commit_message>
Add PDRB geometric decay
</commit_message>
<xml_diff>
--- a/DeskripsiSektor.xlsx
+++ b/DeskripsiSektor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_LASSO\LAS_Simulation_Jateng\I-O_Analysis\Regional-Economy---Jawa-Tengah\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy---Jawa-Tengah/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{68BCB2A9-3034-4403-B0F6-B9866D2064DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C2824A85-1FF2-4FE4-93CA-E4661EDCEF1F}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="9960" xr2:uid="{C2824A85-1FF2-4FE4-93CA-E4661EDCEF1F}"/>
   </bookViews>
   <sheets>
     <sheet name="DeskripsiSektor" sheetId="1" r:id="rId1"/>
@@ -726,17 +726,17 @@
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:J67"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="11.08203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="75.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.58203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="75.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.59765625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.69921875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.08203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="55.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="55.296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">

</xml_diff>